<commit_message>
documentation and tc update
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-30_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-30_Test_Cases.xlsx
@@ -1434,7 +1434,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1443,7 +1443,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>SPM-30 fixtures loaded: 'SPM30 Nusantara Developer Meetup' (organiser Budi Santoso, Nusantara Tech Labs) is Submitted with no coordinator.
-Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
+Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
+Data reset: Changes data (assigns the event). TC09 and TC10 continue from this result, so reset only after TC10: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1599,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1607,7 +1608,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>TC08 completed: Daniel Tan is assigned to 'SPM30 Nusantara Developer Meetup'.
-Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
+Data reset: Changes data (adds an equipment requirement). Reset after TC10: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1762,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1769,7 +1771,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>TC08 completed: Daniel Tan is assigned to 'SPM30 Nusantara Developer Meetup'.
-Logged in as Budi Santoso (budi.santoso@nusantaratec.com / password123), the event's organiser.</t>
+Logged in as Budi Santoso (budi.santoso@nusantaratec.com / password123), the event's organiser.
+Data reset: After this case, reset the data TC08 and TC09 changed: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2240,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2246,7 +2249,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>SPM-30 fixtures loaded: 'SPM30 Kirana Regional Offsite' (organiser Faridah Aziz) is Under review with coordinator Priya Raj.
-Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
+Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
+Data reset: Changes data (reassigns the event). TC14 continues from this result, so reset only after TC14: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2406,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2410,7 +2414,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>TC13 completed: 'SPM30 Kirana Regional Offsite' reassigned from Priya Raj to Joel Fernandez.</t>
+          <t>TC13 completed: 'SPM30 Kirana Regional Offsite' reassigned from Priya Raj to Joel Fernandez.
+Data reset: After this case, reset the data TC13 changed: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2569,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2573,7 +2578,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>SPM-30 fixtures loaded: 'SPM30 Nusantara Product Launch' (organiser Sari Widodo) is Under review with coordinator Daniel Tan.
-Logged in as Nadia Rahman (nadia.rahman@connectsphere.com / password123), Event Operations Manager.</t>
+Logged in as Nadia Rahman (nadia.rahman@connectsphere.com / password123), Event Operations Manager.
+Data reset: Changes data (reassigns the event). After this case, reset it: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2735,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2738,7 +2744,8 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>SPM-30 fixtures loaded: 'SPM30 Anchorpoint Partner Briefing' is Confirmed with coordinator Joel Fernandez; 'SPM30 Civic Trust Workshop' is Postponed with coordinator Arif Mansor.
-Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
+Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
+Data reset: Changes data (reassigns both events). After this case, reset them: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3566,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3569,7 +3576,8 @@
         <is>
           <t>Run on a Neon branch or local database, not the shared one.
 Every event in the 'Awaiting assignment' list has been assigned, so no submitted event is unassigned.
-Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
+Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
+Data reset: Changes data on the branch (every submitted event gets a coordinator, including base-seed events the SPM-30 reset does not cover). Afterwards, reset that branch with `npx prisma db seed` then `npm run fixtures:spm30`, or delete the branch. Never reseed the shared database.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated tc and db seeding
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-30_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-30_Test_Cases.xlsx
@@ -1434,7 +1434,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1442,7 +1442,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Nusantara Developer Meetup' (organiser Budi Santoso, Nusantara Tech Labs) is Submitted with no coordinator.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Nusantara Developer Meetup' (organiser Budi Santoso, Nusantara Tech Labs) is Submitted with no coordinator.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
 Data reset: Changes data (assigns the event). TC09 and TC10 continue from this result, so reset only after TC10: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
@@ -1476,7 +1477,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="85" customHeight="1">
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1484,7 +1485,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A success message confirming the assignment is shown.
+          <t>The message 'Daniel Tan is now the coordinator for "SPM30 Nusantara Developer Meetup". It has moved to Under review.' is shown.
 'SPM30 Nusantara Developer Meetup' disappears from the 'Awaiting assignment' list.
 After reloading the event page, the status badge shows 'Under review' (previously 'Submitted') and the 'Details' card shows Coordinator 'Daniel Tan'.</t>
         </is>
@@ -1784,7 +1785,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events'
+          <t>1. Click 'My Events' in the sidebar
 2. Open 'SPM30 Nusantara Developer Meetup'</t>
         </is>
       </c>
@@ -1922,7 +1923,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1930,7 +1931,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Meridian Client Forum' (owned by James Koh, Meridian Financial Group) is Confirmed with coordinator Daniel Tan.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Meridian Client Forum' (owned by James Koh, Meridian Financial Group) is Confirmed with coordinator Daniel Tan.
 Logged in as Rachel Ng (rachel.ng@meridianfina.com / password123), another organiser at Meridian Financial Group.</t>
         </is>
       </c>
@@ -1943,7 +1945,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events'
+          <t>1. Click 'My Events' in the sidebar
 2. Open 'SPM30 Meridian Client Forum'</t>
         </is>
       </c>
@@ -2081,7 +2083,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2089,7 +2091,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Meridian Client Forum' is Confirmed, registration enabled, coordinator Daniel Tan.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Meridian Client Forum' is Confirmed, registration enabled, coordinator Daniel Tan.
 Logged in as an Attendee (lee.wei.ming@example.com / password123).</t>
         </is>
       </c>
@@ -2240,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2248,13 +2251,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Kirana Regional Offsite' (organiser Faridah Aziz) is Under review with coordinator Priya Raj.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Kirana Regional Offsite' (organiser Faridah Aziz) is Under review with coordinator Priya Raj.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
 Data reset: Changes data (reassigns the event). TC14 continues from this result, so reset only after TC14: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
+    <row r="4" ht="112" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2264,9 +2268,9 @@
         <is>
           <t>1. Click 'All Events'
 2. Open 'SPM30 Kirana Regional Offsite'
-3. Choose the option to change the coordinator
-4. Select 'Joel Fernandez'
-5. Confirm the change
+3. In the 'Change coordinator' card, choose 'Joel Fernandez' from the dropdown
+4. Click 'Reassign'
+5. Click 'Reassign' in the 'Reassign this event?' confirmation
 6. Reload the page</t>
         </is>
       </c>
@@ -2283,7 +2287,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2291,7 +2295,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A success message confirming the reassignment is shown.
+          <t>The confirmation says the event moves from Priya Raj to Joel Fernandez.
+The message 'Reassigned from Priya Raj to Joel Fernandez.' is shown.
 After reloading, the 'Details' card shows Coordinator 'Joel Fernandez'.
 The event status is unchanged (Under review).</t>
         </is>
@@ -2569,7 +2574,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2577,13 +2582,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Nusantara Product Launch' (organiser Sari Widodo) is Under review with coordinator Daniel Tan.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Nusantara Product Launch' (organiser Sari Widodo) is Under review with coordinator Daniel Tan.
 Logged in as Nadia Rahman (nadia.rahman@connectsphere.com / password123), Event Operations Manager.
 Data reset: Changes data (reassigns the event). After this case, reset it: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="112" customHeight="1">
+    <row r="4" ht="125.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2592,11 +2598,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Assignments' in the sidebar
-2. Switch to the view listing events that already have a coordinator
+2. Click the 'Assigned' tab
 3. Find the row for 'SPM30 Nusantara Product Launch'
-4. Choose 'Hui Shan Neo' as the new coordinator
-5. Confirm the change
-6. Click 'All Events' and open 'SPM30 Nusantara Product Launch'</t>
+4. In that row's dropdown, choose 'Hui Shan Neo'
+5. Click 'Reassign' in that row
+6. Click 'Reassign' in the 'Reassign this event?' confirmation
+7. Click 'All Events' and open 'SPM30 Nusantara Product Launch'</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2619,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2620,7 +2627,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A success message confirming the reassignment is shown.
+          <t>The message '"SPM30 Nusantara Product Launch" has been reassigned from Daniel Tan to Hui Shan Neo.' is shown.
 The event page shows Coordinator 'Hui Shan Neo'.
 The event status is unchanged (Under review).</t>
         </is>
@@ -2735,7 +2742,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2743,13 +2750,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Anchorpoint Partner Briefing' is Confirmed with coordinator Joel Fernandez; 'SPM30 Civic Trust Workshop' is Postponed with coordinator Arif Mansor.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Anchorpoint Partner Briefing' is Confirmed with coordinator Joel Fernandez; 'SPM30 Civic Trust Workshop' is Postponed with coordinator Arif Mansor.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
 Data reset: Changes data (reassigns both events). After this case, reset them: run `npm run fixtures:spm30` from the project folder.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2759,9 +2767,9 @@
         <is>
           <t>1. Click 'All Events'
 2. Open 'SPM30 Anchorpoint Partner Briefing'
-3. Change the coordinator to 'Arif Mansor' and confirm
-4. Open 'SPM30 Civic Trust Workshop'
-5. Change the coordinator to 'Hui Shan Neo' and confirm</t>
+3. In the 'Change coordinator' card, choose 'Arif Mansor', click 'Reassign', then 'Reassign' in the confirmation
+4. Click 'All Events' and open 'SPM30 Civic Trust Workshop'
+5. In the 'Change coordinator' card, choose 'Hui Shan Neo', click 'Reassign', then 'Reassign' in the confirmation</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2908,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2908,7 +2916,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Harbourline Claims Training' is Completed (Priya Raj), 'SPM30 Pearl Delta Supplier Forum' is Cancelled (Joel Fernandez), 'SPM30 Selaras Overnight Field Day' is Rejected (Priya Raj).
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Harbourline Claims Training' is Completed (Priya Raj), 'SPM30 Pearl Delta Supplier Forum' is Cancelled (Joel Fernandez), 'SPM30 Selaras Overnight Field Day' is Rejected (Priya Raj).
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -2922,10 +2931,10 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click 'All Events'
-2. Open 'SPM30 Harbourline Claims Training' and look for an option to change the coordinator
-3. Open 'SPM30 Pearl Delta Supplier Forum' and look for an option to change the coordinator
-4. Open 'SPM30 Selaras Overnight Field Day' and look for an option to change the coordinator
-5. Click 'Assignments' and check whether any of these three events are listed</t>
+2. Open 'SPM30 Harbourline Claims Training' and look for a 'Change coordinator' card
+3. Open 'SPM30 Pearl Delta Supplier Forum' and look for a 'Change coordinator' card
+4. Open 'SPM30 Selaras Overnight Field Day' and look for a 'Change coordinator' card
+5. Click 'Assignments', open the 'Assigned' tab, and check whether any of these three events are listed</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2950,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2949,8 +2958,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>No option to change the coordinator is shown on any of the three events.
-None of them appear on the Assignments page.
+          <t>None of the three events shows a 'Change coordinator' card.
+None of them appear on either Assignments tab.
 Each still shows its original coordinator.</t>
         </is>
       </c>
@@ -3037,7 +3046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3062,148 +3071,49 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="71.5" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>NOTE: SPM-30 is not implemented yet. The Assignments page (src/app/assignments/page.tsx) is a 'not built yet' placeholder and there is no assignment endpoint. Steps follow the S-28 Assignment Queue mockup (design/mockups/AssignmentQueue.dc.html) and must be re-checked against the built UI (button labels, messages, reassign controls).</t>
+          <t>NOTE: Test data comes from scripts/seed-spm30.ts (npm run fixtures:spm30). It only deletes and recreates events whose seed key starts with 'spm30_'; the rest of the database is untouched. Run it before a full pass, and wherever a case's 'Data reset' line says to.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>NOTE: Test data comes from scripts/seed-spm30.ts (npm run fixtures:spm30). It only deletes and recreates events whose seed key starts with 'spm30_'; the rest of the database is untouched. Run it before a full pass (TC01-TC19 run in order from fresh fixtures) and again afterwards to reset.</t>
+          <t>NOTE: TC20 (empty state) runs on the shared database. It assigns the two base-seed events that start in the queue, so it must run last and be followed by `npm run fixtures:spm30`, which puts them back (if another story has since moved one past Under review, the script leaves it and says so; `-- --restore-queue` forces it). If the queue holds any other event (e.g. one a teammate created in the app), TC20 says to stop rather than assign it, because the script cannot restore it.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>NOTE: TC20 (empty state) needs zero unassigned submitted events in the whole database, which on the shared database means assigning base-seed events such as 'Nusantara Developer Summit'. The fixture script does not restore those. Run TC20 on a Neon branch or local database.</t>
+          <t>NOTE: Organisers from an unrelated company not seeing the event is covered by SPM-31 (visibility), so it is not repeated here.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n"/>
     </row>
-    <row r="5" ht="31" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>NOTE: Organisers from an unrelated company not seeing the event is covered by SPM-31 (visibility), so it is not repeated here.</t>
+          <t>OPEN: Notifications are written on assignment (new coordinator) and reassignment (new and previous coordinator), but there are no test cases for them yet because the Notifications page (S-04, SPM-53) is still a placeholder. Add them once SPM-53 is built.</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: Only the Event Operations Manager can assign or reassign a coordinator (no self-assignment).</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: Assigning a coordinator moves the event from Submitted to Under review (TC08). So a Submitted event never has a coordinator, and filtering the Ops Manager dashboard's 'Awaiting assignment' section on status Submitted is enough.</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: Reassignment is available from both the event detail page (TC13) and the Assignments page (TC15). The mockup has no Assignments view for already-assigned events yet; re-check TC15's steps once built.</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="44.5" customHeight="1">
-      <c r="A9" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: Events can be reassigned in any active status (Under review, Approved, Planning, Confirmed, Postponed), not Completed, Cancelled or Rejected (TC16, TC17).</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n"/>
-    </row>
-    <row r="10" ht="44.5" customHeight="1">
-      <c r="A10" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: The owning organiser and organisers from the same client organisation see the assigned coordinator at any non-draft status, with 'Not yet assigned' shown until then (TC06, TC10, TC11).</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n"/>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: Remove the 'any coordinator can manage an unassigned event' allowance (TC07). This requires changing isAssignedCoordinator in src/lib/permissions.ts and updating docs/PERMISSIONS.md ('Assigned' relationship and Open items).</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n"/>
-    </row>
-    <row r="12" ht="71.5" customHeight="1">
-      <c r="A12" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: On assignment the new coordinator is notified; on reassignment both the new and previous coordinators are notified; the organiser is not notified. No test cases yet because the Notifications page (S-04, SPM-53) is still a placeholder, so a tester cannot see notifications on screen. Add them once SPM-53 is built.</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n"/>
-    </row>
-    <row r="13" ht="85" customHeight="1">
-      <c r="A13" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>RESOLVED 2026-09-28: The mockup's 'Coordinator workload' panel is not a requirement. Customer clarification #93: choosing a coordinator 'is up to Event Operations Manager, they have their own SOP which is handled outside of the system'. #92: a coordinator can be assigned to multiple events concurrently (no cap). No Jira story covers it. Out of scope for SPM-30; no test cases.</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="n"/>
-    </row>
-    <row r="14" ht="112" customHeight="1">
-      <c r="A14" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>CONFIRMED by customer clarifications (docs/discussions/20260916): #94 and #101 - only the Event Operations Manager assigns and reassigns, as a separate role, and reassignment approval happens outside the system; #95 - no acceptance step, the assignment takes effect immediately (TC09); #81 - organisers in the same client organisation may view each other's events (TC11); #117 - the Ops Manager must be able to identify newly submitted events needing assignment, without a notification per submission (TC01, TC02).</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3243,7 +3153,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3251,7 +3161,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Straits Journal Club' is Under review with coordinator Joel Fernandez.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Straits Journal Club' is Under review with coordinator Joel Fernandez.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -3266,8 +3177,7 @@
         <is>
           <t>1. Click 'All Events'
 2. Open 'SPM30 Straits Journal Club'
-3. Choose the option to change the coordinator
-4. Select 'Joel Fernandez' (the current coordinator)</t>
+3. In the 'Change coordinator' card, choose 'Joel Fernandez' (the current coordinator) from the dropdown</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3193,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3291,7 +3201,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The confirm button is disabled, or a message says Joel Fernandez is already the assigned coordinator.
+          <t>The message 'Joel Fernandez is already the assigned coordinator.' appears under the dropdown.
+The 'Reassign' button stays disabled.
 The coordinator remains 'Joel Fernandez'.</t>
         </is>
       </c>
@@ -3405,7 +3316,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3413,7 +3324,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Straits Journal Club' is Under review with coordinator Joel Fernandez (organiser Raj Kumar).</t>
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Straits Journal Club' is Under review with coordinator Joel Fernandez (organiser Raj Kumar).</t>
         </is>
       </c>
     </row>
@@ -3426,9 +3338,9 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Log in as Joel Fernandez (joel.fernandez@connectsphere.com / password123)
-2. Open 'SPM30 Straits Journal Club' and look for an option to change the coordinator
+2. Click 'All Events', open 'SPM30 Straits Journal Club' and look for a 'Change coordinator' card
 3. Log out and log in as Raj Kumar (raj.kumar@straitsmedic.com / password123)
-4. Open 'SPM30 Straits Journal Club' and look for an option to change the coordinator</t>
+4. Click 'My Events', open 'SPM30 Straits Journal Club' and look for a 'Change coordinator' card</t>
         </is>
       </c>
     </row>
@@ -3452,8 +3364,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Neither user sees any option to assign or change the coordinator.
-The Coordinator row shows 'Joel Fernandez' as read-only text.</t>
+          <t>Neither user sees a 'Change coordinator' card or any other way to assign or change the coordinator.
+The 'Details' card shows Coordinator 'Joel Fernandez' as read-only text.</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3478,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="152.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3574,14 +3486,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run on a Neon branch or local database, not the shared one.
-Every event in the 'Awaiting assignment' list has been assigned, so no submitted event is unassigned.
+          <t>Test data freshly loaded: run `npm run fixtures:spm30` from the project folder just before this case.
+Run this case last in the pass: it assigns every event waiting for a coordinator, including two base-seed events other stories' test cases rely on.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).
-Data reset: Changes data on the branch (every submitted event gets a coordinator, including base-seed events the SPM-30 reset does not cover). Afterwards, reset that branch with `npx prisma db seed` then `npm run fixtures:spm30`, or delete the branch. Never reseed the shared database.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="17.5" customHeight="1">
+Data reset: after this case, run `npm run fixtures:spm30` from the project folder. It resets the SPM30 events and puts 'Nusantara Developer Summit' and 'Meridian Graduate Recruitment Evening' back to Submitted with no coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3589,11 +3501,14 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Assignments' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Click 'Assignments' in the sidebar
+2. Check the 'Awaiting assignment' list contains only the four expected events (see test data); if it lists any other event, stop and do not assign it
+3. For each event in the list, choose 'Daniel Tan' in its 'Assign to' dropdown and click 'Assign'
+4. Reload the page</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3601,11 +3516,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Unassigned submitted events: 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Expected queue before assigning (4 events): SPM30 Nusantara Developer Meetup, SPM30 Meridian Graduate Evening, Nusantara Developer Summit, Meridian Graduate Recruitment Evening | Coordinator for all: Daniel Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3613,7 +3528,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>An empty-state message is shown saying there are no events awaiting assignment.
+          <t>After the last assignment, and again after reloading, the 'Awaiting assignment' tab shows the message 'No events are awaiting assignment' with 'Every submitted event has a coordinator.'
 No table rows and no error are shown.</t>
         </is>
       </c>
@@ -3727,7 +3642,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3735,12 +3650,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures freshly loaded (npm run fixtures:spm30).
+          <t>Test data freshly loaded: run `npm run fixtures:spm30` from the project folder just before this case.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123), Event Operations Manager.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="17.5" customHeight="1">
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3748,7 +3663,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Assignments' in the sidebar</t>
+          <t>1. Click 'Assignments' in the sidebar
+2. Click 'SPM30 Meridian Graduate Evening' in the list to open it</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3680,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="98.5" customHeight="1">
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3772,10 +3688,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The 'Awaiting assignment' table shows 'SPM30 Nusantara Developer Meetup' and 'SPM30 Meridian Graduate Evening' with their client, date and how long they have been waiting.
+          <t>The 'Awaiting assignment' table shows 'SPM30 Nusantara Developer Meetup' and 'SPM30 Meridian Graduate Evening' with their client, date and how long they have been waiting. Base-seed events that are also submitted with no coordinator (e.g. 'Nusantara Developer Summit', 'Meridian Graduate Recruitment Evening') may appear too.
 'SPM30 Kirana Regional Offsite' (already has a coordinator) is not listed.
 'SPM30 Draft Investor Update' (draft) is not listed.
-Every row shown has status Submitted.</t>
+The opened event's page shows the 'Submitted' status badge next to its title, and Coordinator 'Not yet assigned'.</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3804,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3896,7 +3812,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures freshly loaded.
+          <t>Test data freshly loaded: run `npm run fixtures:spm30` from the project folder just before this case.
 Logged in as Nadia Rahman (nadia.rahman@connectsphere.com / password123), Event Operations Manager.</t>
         </is>
       </c>
@@ -4214,7 +4130,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4222,7 +4138,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -4374,7 +4290,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4382,7 +4298,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -4421,7 +4338,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The 'Assign' button is disabled, or a validation message asking to choose a coordinator is shown.
+          <t>The 'Assign' button stays disabled while 'Choose a coordinator' is selected.
 The event stays in the 'Awaiting assignment' list with status Submitted.</t>
         </is>
       </c>
@@ -4535,7 +4452,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4543,7 +4460,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
 Logged in as James Koh (james.koh@meridianfina.com / password123), the event's organiser.</t>
         </is>
       </c>
@@ -4556,7 +4474,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events'
+          <t>1. Click 'My Events' in the sidebar
 2. Open 'SPM30 Meridian Graduate Evening'</t>
         </is>
       </c>
@@ -4694,7 +4612,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4702,7 +4620,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-30 fixtures loaded: 'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
+          <t>Test data loaded: run `npm run fixtures:spm30` from the project folder if it has not been run for this test pass.
+'SPM30 Meridian Graduate Evening' is Submitted with no coordinator.
 Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), Event Coordinator.</t>
         </is>
       </c>
@@ -4734,7 +4653,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="85" customHeight="1">
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4744,7 +4663,7 @@
         <is>
           <t>The event does not appear under 'Awaiting your review' on Daniel Tan's dashboard.
 The event details can be viewed and show Coordinator 'Not yet assigned'.
-No options to add or edit equipment requirements, or to change the event's status, are available.</t>
+The Equipment tab shows 'Only the coordinator assigned to this event can view and manage its equipment requirements.' and no options to add or edit equipment.</t>
         </is>
       </c>
     </row>

</xml_diff>